<commit_message>
Added new RDF data schemes and visual schemes for environment-table36-38, and fixed XLSX spreadsheets for environment-table36-37
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table36.xlsx
+++ b/sources/table_normalization/xlsx/environment-table36.xlsx
@@ -148,7 +148,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -330,12 +330,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -345,37 +360,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -877,122 +877,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.5">
-      <c r="A1" s="10"/>
-      <c r="B1" s="11"/>
-      <c r="C1" s="5" t="s">
+      <c r="A1" s="13"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="5" t="s">
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="5" t="s">
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="5" t="s">
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="7"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="12"/>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="12"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="16" t="s">
+      <c r="A2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="16" t="s">
+      <c r="D2" s="18"/>
+      <c r="E2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="17"/>
-      <c r="G2" s="16" t="s">
+      <c r="F2" s="18"/>
+      <c r="G2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="17"/>
-      <c r="I2" s="16" t="s">
+      <c r="H2" s="18"/>
+      <c r="I2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="17"/>
-      <c r="K2" s="16" t="s">
+      <c r="J2" s="18"/>
+      <c r="K2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="17"/>
-      <c r="M2" s="16" t="s">
+      <c r="L2" s="18"/>
+      <c r="M2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="17"/>
-      <c r="O2" s="16" t="s">
+      <c r="N2" s="18"/>
+      <c r="O2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="16" t="s">
+      <c r="P2" s="18"/>
+      <c r="Q2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="R2" s="17"/>
+      <c r="R2" s="18"/>
     </row>
     <row r="3" spans="1:18" ht="29">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="18" t="s">
+      <c r="K3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="L3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="18" t="s">
+      <c r="M3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="O3" s="18" t="s">
+      <c r="O3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="18" t="s">
+      <c r="P3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="Q3" s="18" t="s">
+      <c r="Q3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="R3" s="18" t="s">
+      <c r="R3" s="7" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1494,11 +1494,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A1:B2"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="G1:J1"/>
     <mergeCell ref="K1:N1"/>
@@ -1511,6 +1506,11 @@
     <mergeCell ref="M2:N2"/>
     <mergeCell ref="O2:P2"/>
     <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A1:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>